<commit_message>
added user storys and requirements
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Elektrotechnik\6. Semester\Prozessortechnik\Projekt\Orga\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Documents\Prozessortechink_projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEC5D7D-1CD0-4A80-AAC7-D3A8FEAFFA59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853F9012-BEFC-416E-AA7A-3061420F157F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="156">
   <si>
     <t>User Story ID</t>
   </si>
@@ -61,6 +61,9 @@
     <t>Traceability Anforderungen</t>
   </si>
   <si>
+    <t>US_G5_2</t>
+  </si>
+  <si>
     <t>US_G5_3</t>
   </si>
   <si>
@@ -136,72 +139,12 @@
     <t>A_G5_5</t>
   </si>
   <si>
-    <t>A_G5_6</t>
-  </si>
-  <si>
-    <t>A_G5_7</t>
-  </si>
-  <si>
-    <t>A_G5_8</t>
-  </si>
-  <si>
-    <t>A_G5_9</t>
-  </si>
-  <si>
-    <t>A_G5_10</t>
-  </si>
-  <si>
-    <t>A_G5_11</t>
-  </si>
-  <si>
-    <t>A_G5_12</t>
-  </si>
-  <si>
-    <t>A_G5_13</t>
-  </si>
-  <si>
-    <t>A_G5_14</t>
-  </si>
-  <si>
-    <t>A_G5_15</t>
-  </si>
-  <si>
-    <t>A_G5_16</t>
-  </si>
-  <si>
     <t>US_G5_4</t>
   </si>
   <si>
     <t>US_G5_5</t>
   </si>
   <si>
-    <t>US_G5_6</t>
-  </si>
-  <si>
-    <t>US_G5_7</t>
-  </si>
-  <si>
-    <t>US_G5_8</t>
-  </si>
-  <si>
-    <t>US_G5_9</t>
-  </si>
-  <si>
-    <t>US_G5_10</t>
-  </si>
-  <si>
-    <t>US_G5_11</t>
-  </si>
-  <si>
-    <t>US_G5_12</t>
-  </si>
-  <si>
-    <t>US_G5_13</t>
-  </si>
-  <si>
-    <t>US_G5_14</t>
-  </si>
-  <si>
     <t>TC_G5_7</t>
   </si>
   <si>
@@ -289,15 +232,6 @@
     <t>negative test</t>
   </si>
   <si>
-    <t xml:space="preserve">Als &lt;Beschreibung Benutzer&gt; will ich &lt;Beschreibung Funktion&gt;, so dass &lt;Beschreibung Nutzen&gt; </t>
-  </si>
-  <si>
-    <t>Gegeben, dass &lt;&gt;, wenn &lt;Beschreibung Aktion&gt;,  dann &lt;Ergebnis der Aktion&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bedingung&gt; muss &lt;Subjekt&gt;&lt;Objekt&gt;&lt;zusätzliche Angaben&gt;&lt;Verb&gt;</t>
-  </si>
-  <si>
     <t>Traceability Architektur</t>
   </si>
   <si>
@@ -361,12 +295,6 @@
     <t>ArchEl_19</t>
   </si>
   <si>
-    <t>Auswahl Seite</t>
-  </si>
-  <si>
-    <t>Wenn die tiefe Seite E auf dem Display angewählt wird, dann muss die Anwedung die Seite E mit der entpsrecheden Soll-Frequenz 82 Hz anzeigen</t>
-  </si>
-  <si>
     <t>Aufwand</t>
   </si>
   <si>
@@ -475,12 +403,6 @@
     <t>failed</t>
   </si>
   <si>
-    <t>Als Gitarrenspieler will ich die Seite zum Stimmen auf dem display wählen, so dass die Seite für die Stimmung klar definiert ist</t>
-  </si>
-  <si>
-    <t>Gegeben, dass auf dem Display die Seiten angezeigt werden, wenn ich als Gitarrenspieler eine Seite auf dem Display auswähle,  dann wird die Seite mit der entsprechenden Soll-Frequenz angezeigt.</t>
-  </si>
-  <si>
     <t>Titel</t>
   </si>
   <si>
@@ -502,29 +424,98 @@
     <t>Projektthema</t>
   </si>
   <si>
+    <t>z.B. 1.0</t>
+  </si>
+  <si>
     <t>Gruppe 1</t>
   </si>
   <si>
-    <t>Audio BPM Erkennung</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>US_G1_1</t>
-  </si>
-  <si>
-    <t>US_G1_2</t>
-  </si>
-  <si>
-    <t>A_G1_1</t>
+    <t>Audio BPM Geschwindigkeitserkennung</t>
+  </si>
+  <si>
+    <t>Der Live-Musiker (Synchronisation)</t>
+  </si>
+  <si>
+    <t>Der DJ (Analog-Mixing)</t>
+  </si>
+  <si>
+    <t>Der Lichttechniker (Show-Automatisierung)</t>
+  </si>
+  <si>
+    <t>Der Embedded-Entwickler (Effizienz &amp; Latenz)</t>
+  </si>
+  <si>
+    <t>Der Fitness-Trainer / Tanzlehrer</t>
+  </si>
+  <si>
+    <t>Als Schlagzeuger in einer Band, die mit vorproduzierten Backing-Tracks arbeitet, möchte ich das aktuelle Tempo des analogen Mixers in Echtzeit auf einem Display sehen, damit ich sofort erkenne, ob wir aus dem Takt geraten, ohne auf ein komplexes Laptop-Setup angewiesen zu sein.</t>
+  </si>
+  <si>
+    <t>Die BPM-Anzeige darf eine maximale Abweichung von ±1 BPM gegenüber dem tatsächlichen Tempo aufweisen und muss sich bei Tempowechseln innerhalb von weniger als 2 Sekunden stabilisieren.</t>
+  </si>
+  <si>
+    <t>Als Vinyl-DJ, der rein analoge Plattenspieler nutzt, möchte ich eine präzise digitale BPM-Anzeige für mein analoges Audiosignal haben, damit ich zwei Tracks schneller und exakter angleichen (Beatmatching) kann, ohne mich nur auf mein Gehör verlassen zu müssen.</t>
+  </si>
+  <si>
+    <t>Das System muss BPM-Werte im Bereich von 60 bis 180 BPM zuverlässig erkennen und den Wert mit mindestens einer Nachkommastelle (z. B. 124.5) auf dem Display ausgeben, um feine Angleichungen zu ermöglichen.</t>
+  </si>
+  <si>
+    <t>Als Lichttechniker bei einem Konzert, möchte ich die BPM der Live-Musik als verlässlichen Zahlenwert ablesen können, damit ich die Geschwindigkeit der Lichteffekte (Stroboskope/Moving Heads) manuell oder halbautomatisch perfekt auf den Rhythmus abstimmen kann.</t>
+  </si>
+  <si>
+    <t>Signalerfassung</t>
+  </si>
+  <si>
+    <t>Der SAP-Algorithmus muss den Grundtakt (Beat) aus dem digitalen Signal in Echtzeit extrahieren.</t>
+  </si>
+  <si>
+    <t>BPM-Analyse</t>
+  </si>
+  <si>
+    <t>Wertebereich</t>
+  </si>
+  <si>
+    <t>Das System muss den berechneten BPM-Wert auf einem integrierten Display (z. B. OLED oder LCD) anzeigen.</t>
+  </si>
+  <si>
+    <t>Informationsausgabe</t>
+  </si>
+  <si>
+    <t>Ein optisches Signal (z. B. eine blinkende LED oder ein Symbol am Display) muss im Takt der Musik aufleuchten.</t>
+  </si>
+  <si>
+    <t>Visueller Feedback</t>
+  </si>
+  <si>
+    <t>Das System muss einen Tempobereich von mindestens 60 bis 180 BPM abdecken.</t>
+  </si>
+  <si>
+    <t>Das System muss ein analoges Audiosignal über einen Line-In (z. B. Klinke) empfangen und mittels ADC für den DSP digitalisieren.</t>
+  </si>
+  <si>
+    <t>Felix Maunz</t>
+  </si>
+  <si>
+    <t>Das Display muss auch unter schwierigen Lichtverhältnissen (dunkle Bühne, bewegtes Licht) aus einer Entfernung von mindestens 1,5 Metern klar lesbar sein und den Takt visuell (z. B. ein blinkendes Display/LED) bestätigen.</t>
+  </si>
+  <si>
+    <t>Als Entwickler von Audio-Hardware, möchte ich die BPM-Berechnung direkt auf einem integrierten DSP durchführen, damit ich eine extrem geringe Latenz erreiche und die Haupt-CPU des Mikrocontrollers für andere Aufgaben (wie das Display-Rendering) entlaste.</t>
+  </si>
+  <si>
+    <t>Die Signalverarbeitung auf dem DSP muss so optimiert sein, dass die CPU-Last des Hauptprozessors für die reine BPM-Berechnung unter 50% bleibt, während das analoge Signal ohne hörbare Verzögerung oder Störung durchgeschleift oder analysiert wird.</t>
+  </si>
+  <si>
+    <t>Als Kursleiter in einem Sportstudio, möchte ich bei jeder beliebigen analogen Audioquelle sofort die BPM sehen, damit ich sicherstellen kann, dass der Musikrhytmus exakt den Vorgaben des Trainingsplans (z. B. 128 BPM für Aerobic) entspricht.</t>
+  </si>
+  <si>
+    <t>Das Gerät muss über eine „Plug-and-Play“-Funktionalität verfügen, bei der nach dem Anstecken des analogen Signals (z. B. Klinke) ohne manuelle Kalibrierung innerhalb von 60 Sekunden ein plausibler BPM-Wert erscheint.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -577,6 +568,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -869,7 +871,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -970,6 +972,36 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1252,58 +1284,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" ht="33.4" x14ac:dyDescent="1">
       <c r="A1" s="18" t="s">
-        <v>146</v>
+        <v>120</v>
       </c>
       <c r="B1" s="19" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+      <c r="A2" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+      <c r="A3" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="39" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+      <c r="A4" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A2" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A3" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A4" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="33.4" x14ac:dyDescent="1">
       <c r="A5" s="20" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="34" thickBot="1" x14ac:dyDescent="0.8">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="33.75" thickBot="1" x14ac:dyDescent="1.05">
       <c r="A6" s="22" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="B6" s="23">
-        <v>46128</v>
+        <v>46133</v>
       </c>
     </row>
   </sheetData>
@@ -1315,22 +1347,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.26953125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.1796875" style="9" customWidth="1"/>
+    <col min="1" max="1" width="13.265625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.1328125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.3984375" style="9" customWidth="1"/>
+    <col min="4" max="4" width="36.1328125" style="9" customWidth="1"/>
     <col min="5" max="6" width="24" style="11" customWidth="1"/>
-    <col min="7" max="7" width="25.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.453125" style="6"/>
+    <col min="7" max="7" width="25.59765625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.3984375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="5" t="s">
@@ -1339,285 +1371,211 @@
       <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="E1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="41" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="7"/>
-    </row>
-    <row r="15" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G15" s="7"/>
+      <c r="B3" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="41" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>152</v>
+      </c>
+      <c r="D5" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="A6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A7" s="42"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="42"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A8" s="42"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="42"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="42"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A10" s="42"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="42"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="42"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" s="42"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="42"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="42"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="42"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A15" s="42"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="42"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1651,418 +1609,305 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.453125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="11.453125" style="6"/>
-    <col min="5" max="5" width="13.26953125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" style="6"/>
-    <col min="7" max="8" width="23.453125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.26953125" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.453125" style="6"/>
+    <col min="1" max="1" width="14.59765625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.3984375" style="9" customWidth="1"/>
+    <col min="3" max="3" width="13.86328125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="11.3984375" style="6"/>
+    <col min="5" max="5" width="13.265625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.3984375" style="6"/>
+    <col min="7" max="8" width="23.3984375" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.265625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.3984375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="5" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A1" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="C1" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="E1" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I1" s="4" t="s">
+      <c r="G1" s="45" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="H1" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="45" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>75</v>
+        <v>27</v>
+      </c>
+      <c r="B2" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>140</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+    </row>
+    <row r="3" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>71</v>
+        <v>28</v>
+      </c>
+      <c r="B3" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>142</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+    </row>
+    <row r="4" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>71</v>
+        <v>29</v>
+      </c>
+      <c r="B4" s="47" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>143</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+    </row>
+    <row r="5" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>71</v>
+        <v>30</v>
+      </c>
+      <c r="B5" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>145</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+    </row>
+    <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>71</v>
+        <v>31</v>
+      </c>
+      <c r="B6" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>147</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A7" s="42"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A8" s="42"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A9" s="42"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A10" s="42"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A11" s="42"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="42"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="42"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="42"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -2073,7 +1918,7 @@
           <x14:formula1>
             <xm:f>LookUp!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C17</xm:sqref>
+          <xm:sqref>C7:C17</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
           <x14:formula1>
@@ -2097,7 +1942,7 @@
           <x14:formula1>
             <xm:f>'User Stories'!$A$2:$A$15</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G17</xm:sqref>
+          <xm:sqref>G2 G7:G17</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
           <x14:formula1>
@@ -2120,201 +1965,201 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="6.453125" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" customWidth="1"/>
-    <col min="4" max="4" width="21.54296875" customWidth="1"/>
-    <col min="5" max="5" width="20.7265625" customWidth="1"/>
-    <col min="6" max="6" width="22.1796875" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375" customWidth="1"/>
+    <col min="3" max="3" width="19.1328125" customWidth="1"/>
+    <col min="4" max="4" width="21.59765625" customWidth="1"/>
+    <col min="5" max="5" width="20.73046875" customWidth="1"/>
+    <col min="6" max="6" width="22.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="C1" s="24" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="D1" s="24"/>
       <c r="E1" s="24"/>
       <c r="F1" s="24"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C2" s="37" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>139</v>
-      </c>
       <c r="F2" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C3" s="38"/>
       <c r="D3" s="16" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B4" s="12"/>
       <c r="C4" s="2" t="s">
-        <v>126</v>
+        <v>102</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B5" s="13" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B6" s="12"/>
       <c r="C6" s="2" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B7" s="12"/>
       <c r="C7" s="2" t="s">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B8" s="12"/>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B9" s="12"/>
       <c r="C9" s="2" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B10" s="12"/>
       <c r="C10" s="14" t="s">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="E12" s="26"/>
       <c r="F12" s="27"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B13" s="14" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="E13" s="29"/>
       <c r="F13" s="30"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B14" s="14" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>134</v>
+        <v>110</v>
       </c>
       <c r="D14" s="31"/>
       <c r="E14" s="32"/>
       <c r="F14" s="33"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B15" s="2" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="32"/>
       <c r="F15" s="33"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="B16" s="14" t="s">
-        <v>122</v>
+        <v>98</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>129</v>
+        <v>105</v>
       </c>
       <c r="D16" s="31"/>
       <c r="E16" s="32"/>
       <c r="F16" s="33"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B17" s="14" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="D17" s="34"/>
       <c r="E17" s="35"/>
       <c r="F17" s="36"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B18" s="14" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B19" s="2" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2332,256 +2177,256 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="19.453125" customWidth="1"/>
-    <col min="3" max="3" width="22.54296875" customWidth="1"/>
+    <col min="2" max="2" width="19.3984375" customWidth="1"/>
+    <col min="3" max="3" width="22.59765625" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.54296875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" customWidth="1"/>
-    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.59765625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="17.3984375" customWidth="1"/>
+    <col min="7" max="7" width="28.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -2612,242 +2457,242 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" customWidth="1"/>
-    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.1796875" customWidth="1"/>
-    <col min="6" max="6" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.73046875" customWidth="1"/>
+    <col min="3" max="3" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.1328125" customWidth="1"/>
+    <col min="6" max="6" width="15.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use Cases erweitert und finalisiert Anforderungen erweitert, Finalisierung TBD (nach Absprache)
Gerne gegenlesen
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Documents\Prozessortechink_projekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://primion-my.sharepoint.com/personal/david_roesch_primion_eu/Documents/Studium/Semester 6/Prozessortechnik/Github/BPM-Detection/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853F9012-BEFC-416E-AA7A-3061420F157F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="13_ncr:1_{853F9012-BEFC-416E-AA7A-3061420F157F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00248610-6FB3-44DA-96C4-CD25799B7A60}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,14 +41,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="182">
   <si>
     <t>User Story ID</t>
   </si>
   <si>
-    <t>US_G5_1</t>
-  </si>
-  <si>
     <t>User  Story Name</t>
   </si>
   <si>
@@ -64,9 +61,6 @@
     <t>US_G5_2</t>
   </si>
   <si>
-    <t>US_G5_3</t>
-  </si>
-  <si>
     <t>Text</t>
   </si>
   <si>
@@ -127,15 +121,6 @@
     <t>A_G5_1</t>
   </si>
   <si>
-    <t>A_G5_2</t>
-  </si>
-  <si>
-    <t>A_G5_3</t>
-  </si>
-  <si>
-    <t>A_G5_4</t>
-  </si>
-  <si>
     <t>A_G5_5</t>
   </si>
   <si>
@@ -448,57 +433,24 @@
     <t>Der Fitness-Trainer / Tanzlehrer</t>
   </si>
   <si>
-    <t>Als Schlagzeuger in einer Band, die mit vorproduzierten Backing-Tracks arbeitet, möchte ich das aktuelle Tempo des analogen Mixers in Echtzeit auf einem Display sehen, damit ich sofort erkenne, ob wir aus dem Takt geraten, ohne auf ein komplexes Laptop-Setup angewiesen zu sein.</t>
-  </si>
-  <si>
-    <t>Die BPM-Anzeige darf eine maximale Abweichung von ±1 BPM gegenüber dem tatsächlichen Tempo aufweisen und muss sich bei Tempowechseln innerhalb von weniger als 2 Sekunden stabilisieren.</t>
-  </si>
-  <si>
     <t>Als Vinyl-DJ, der rein analoge Plattenspieler nutzt, möchte ich eine präzise digitale BPM-Anzeige für mein analoges Audiosignal haben, damit ich zwei Tracks schneller und exakter angleichen (Beatmatching) kann, ohne mich nur auf mein Gehör verlassen zu müssen.</t>
   </si>
   <si>
-    <t>Das System muss BPM-Werte im Bereich von 60 bis 180 BPM zuverlässig erkennen und den Wert mit mindestens einer Nachkommastelle (z. B. 124.5) auf dem Display ausgeben, um feine Angleichungen zu ermöglichen.</t>
-  </si>
-  <si>
     <t>Als Lichttechniker bei einem Konzert, möchte ich die BPM der Live-Musik als verlässlichen Zahlenwert ablesen können, damit ich die Geschwindigkeit der Lichteffekte (Stroboskope/Moving Heads) manuell oder halbautomatisch perfekt auf den Rhythmus abstimmen kann.</t>
   </si>
   <si>
-    <t>Signalerfassung</t>
-  </si>
-  <si>
-    <t>Der SAP-Algorithmus muss den Grundtakt (Beat) aus dem digitalen Signal in Echtzeit extrahieren.</t>
-  </si>
-  <si>
-    <t>BPM-Analyse</t>
-  </si>
-  <si>
-    <t>Wertebereich</t>
-  </si>
-  <si>
     <t>Das System muss den berechneten BPM-Wert auf einem integrierten Display (z. B. OLED oder LCD) anzeigen.</t>
   </si>
   <si>
-    <t>Informationsausgabe</t>
-  </si>
-  <si>
     <t>Ein optisches Signal (z. B. eine blinkende LED oder ein Symbol am Display) muss im Takt der Musik aufleuchten.</t>
   </si>
   <si>
-    <t>Visueller Feedback</t>
-  </si>
-  <si>
-    <t>Das System muss einen Tempobereich von mindestens 60 bis 180 BPM abdecken.</t>
-  </si>
-  <si>
     <t>Das System muss ein analoges Audiosignal über einen Line-In (z. B. Klinke) empfangen und mittels ADC für den DSP digitalisieren.</t>
   </si>
   <si>
     <t>Felix Maunz</t>
   </si>
   <si>
-    <t>Das Display muss auch unter schwierigen Lichtverhältnissen (dunkle Bühne, bewegtes Licht) aus einer Entfernung von mindestens 1,5 Metern klar lesbar sein und den Takt visuell (z. B. ein blinkendes Display/LED) bestätigen.</t>
-  </si>
-  <si>
     <t>Als Entwickler von Audio-Hardware, möchte ich die BPM-Berechnung direkt auf einem integrierten DSP durchführen, damit ich eine extrem geringe Latenz erreiche und die Haupt-CPU des Mikrocontrollers für andere Aufgaben (wie das Display-Rendering) entlaste.</t>
   </si>
   <si>
@@ -509,13 +461,139 @@
   </si>
   <si>
     <t>Das Gerät muss über eine „Plug-and-Play“-Funktionalität verfügen, bei der nach dem Anstecken des analogen Signals (z. B. Klinke) ohne manuelle Kalibrierung innerhalb von 60 Sekunden ein plausibler BPM-Wert erscheint.</t>
+  </si>
+  <si>
+    <t>Der DSP-Algorithmus muss den Grundtakt (Beat) aus dem digitalen Signal nahezu in Echtzeit extrahieren(maximale Latenz 5 Sekunden).</t>
+  </si>
+  <si>
+    <t>Das System soll signalisieren, wenn keine zur Auswertung verwendbaren Daten am DSP anliegen (Break Part)</t>
+  </si>
+  <si>
+    <t>US_G5_6</t>
+  </si>
+  <si>
+    <t>US_G1_1</t>
+  </si>
+  <si>
+    <t>US_G1_2</t>
+  </si>
+  <si>
+    <t>US_G1_3</t>
+  </si>
+  <si>
+    <t>US_G1_4</t>
+  </si>
+  <si>
+    <t>US_G1_5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das System muss BPM-Werte im Bereich von 60 bis 180 BPM zuverlässig erkennen und den Wert mit mindestens einer Nachkommastelle (z. B. 124.5) auf dem Display ausgeben, um feine Angleichungen zu ermöglichen. </t>
+  </si>
+  <si>
+    <t>Das Display muss auch unter schwierigen Lichtverhältnissen (dunkle Bühne, bewegtes Licht) aus einer Entfernung von maximal 1,5 Metern klar lesbar sein und den Takt visuell (z. B. ein blinkendes Display/LED) bestätigen.</t>
+  </si>
+  <si>
+    <t>Die BPM-Anzeige darf eine maximale Abweichung von ±1 BPM gegenüber dem tatsächlichen Tempo aufweisen und muss sich bei Tempowechseln innerhalb von weniger als 5 Sekunden stabilisieren.</t>
+  </si>
+  <si>
+    <t>Als Schlagzeuger in einer Band, die mit vorproduzierten Backing-Tracks arbeitet, möchte ich das aktuelle Tempo des analogen Mixers in Echtzeit auf einem Display sehen, damit ich erkenne, ob wir aus dem Takt geraten, ohne auf ein komplexes Laptop-Setup angewiesen zu sein.</t>
+  </si>
+  <si>
+    <t>Der DJ (Getaktete Effekte)</t>
+  </si>
+  <si>
+    <t>Als Vinyl-DJ, der rein analoge Plattenspieler nutzt um House und Techno aufzulegen, möchte ich eine präzise digitale BPM-Anzeige für mein analoges Audiosignal haben, damit ich meine externen Effektgeräte an die BPM angleichen kann. Gerade in den Breakparts ohne Drums ist der Einsatz von Effekten ein wichtiger Bestandteil des Mixings</t>
+  </si>
+  <si>
+    <t>A_G1_1</t>
+  </si>
+  <si>
+    <t>A_G1_2</t>
+  </si>
+  <si>
+    <t>A_G1_7</t>
+  </si>
+  <si>
+    <t>A_G1_3</t>
+  </si>
+  <si>
+    <t>A_G1_4</t>
+  </si>
+  <si>
+    <t>US_G1_6</t>
+  </si>
+  <si>
+    <t>A_G1_5</t>
+  </si>
+  <si>
+    <t>A_G1_6</t>
+  </si>
+  <si>
+    <t>A_G1_8</t>
+  </si>
+  <si>
+    <t>A_G1_9</t>
+  </si>
+  <si>
+    <t>Das System muss innerhalb von 60 Sekunden nach Start der Energieversorgung selbstständig und ohne zusätzliche Betätigungen durch den User "ready to use" sein</t>
+  </si>
+  <si>
+    <t>Das System muss zwischen keinen Daten (kein Audiosignal) und keinen verwertbaren Daten (keine getaktete Musik, andere Audiosignale) unterscheiden</t>
+  </si>
+  <si>
+    <t>A_G1_10</t>
+  </si>
+  <si>
+    <t>A_G1_11</t>
+  </si>
+  <si>
+    <t>Das System soll den letzten ausgewerteten BPM-Wert solange anzeigen bis entweder eine neue Auswertung erfolgt ist oder das Audiosignal für mehr als 10 Sekunden unterbrochen wurde</t>
+  </si>
+  <si>
+    <t>Das System soll , wenn das Audiosignal für mehr als 10 Sekunden unterbrochen wurde, den Live Wert auf 0 BPM setzen und den letzten gemessenen Wert in einer Ecke des Displays kleingedruckt anzeigen</t>
+  </si>
+  <si>
+    <t>Funktional</t>
+  </si>
+  <si>
+    <t>Nicht-Funktional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das System muss bei anliegenden Audiodaten, die nicht auswertbar sind den letzten erfassten Wert weiterhin auf dem Display anzeigen, aber visuell darauf hinweisen, dass dieser Wert nicht mehr live gemessen wurde </t>
+  </si>
+  <si>
+    <t>Das System muss den gemessenen BPM-Wert auf 1/10 BPM genau anzeigen</t>
+  </si>
+  <si>
+    <t>Das System muss einen Tempobereich von mindestens 60 bis 180 BPM (Beats Per Minute) abdecken.</t>
+  </si>
+  <si>
+    <t>A_G1_12</t>
+  </si>
+  <si>
+    <t>A_G1_13</t>
+  </si>
+  <si>
+    <t>Das System muss auf der bereitgestellten Hardware (STM32F746G-DISCO) funktionieren ohne diese zu überlasten</t>
+  </si>
+  <si>
+    <t>US_G5_1\2\3\5\6</t>
+  </si>
+  <si>
+    <t>Das System muss 4\4 Takte mit durchgehender Kickdrum erkennen können</t>
+  </si>
+  <si>
+    <t>US_G5_3\6</t>
+  </si>
+  <si>
+    <t>US_G5_1\3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -579,6 +657,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -871,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -928,6 +1012,24 @@
     <xf numFmtId="14" fontId="6" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -973,35 +1075,23 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1018,6 +1108,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1284,55 +1378,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+    <row r="1" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A1" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A2" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B2" s="21" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A3" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="33.4" x14ac:dyDescent="1">
-      <c r="A2" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="33.4" x14ac:dyDescent="1">
-      <c r="A3" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="B3" s="39" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A4" s="20" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="33.4" x14ac:dyDescent="1">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A5" s="20" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="33.75" thickBot="1" x14ac:dyDescent="1.05">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="22" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B6" s="23">
         <v>46133</v>
@@ -1346,236 +1440,181 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.265625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.1328125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.3984375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.1328125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="9" customWidth="1"/>
     <col min="5" max="6" width="24" style="11" customWidth="1"/>
-    <col min="7" max="7" width="25.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.3984375" style="6"/>
+    <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="C2" s="41" t="s">
-        <v>135</v>
-      </c>
-      <c r="D2" s="41" t="s">
+      <c r="D3" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F2" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>131</v>
-      </c>
-      <c r="C3" s="41" t="s">
+      <c r="D5" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="E5" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>132</v>
-      </c>
-      <c r="C4" s="41" t="s">
+      <c r="D6" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="41" t="s">
-        <v>151</v>
-      </c>
-      <c r="E4" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A5" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="41" t="s">
-        <v>133</v>
-      </c>
-      <c r="C5" s="41" t="s">
+      <c r="E6" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="C7" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="E5" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>134</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>154</v>
-      </c>
-      <c r="D6" s="41" t="s">
-        <v>155</v>
-      </c>
-      <c r="E6" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A7" s="42"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="42"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" s="42"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="42"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" s="42"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="42"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" s="42"/>
-      <c r="B10" s="42"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="42"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A11" s="42"/>
-      <c r="B11" s="42"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="42"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A12" s="42"/>
-      <c r="B12" s="42"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="42"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" s="42"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="42"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A14" s="42"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="42"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" s="42"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="42"/>
+      <c r="D7" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D12" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1587,17 +1626,17 @@
           <x14:formula1>
             <xm:f>LookUp!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E15</xm:sqref>
+          <xm:sqref>E2:E3 E4:E15</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
             <xm:f>LookUp!$C$2:$C$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F15</xm:sqref>
+          <xm:sqref>F2:F3 F4:F15</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
-            <xm:f>Anforderungen!$A$2:$A$17</xm:f>
+            <xm:f>Anforderungen!$A$2:$A$23</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
         </x14:dataValidation>
@@ -1609,307 +1648,351 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.3984375" style="9" customWidth="1"/>
-    <col min="3" max="3" width="13.86328125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="11.3984375" style="6"/>
-    <col min="5" max="5" width="13.265625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.3984375" style="6"/>
-    <col min="7" max="8" width="23.3984375" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.3984375" style="6"/>
+    <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="48" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="6"/>
+    <col min="7" max="7" width="23.42578125" style="50" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A1" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="46" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="E1" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="45" t="s">
+      <c r="F1" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="G1" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="45" t="s">
+      <c r="H1" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="45" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="45" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="45" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="45" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="45" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="45" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>177</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>171</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="47" t="s">
-        <v>149</v>
-      </c>
-      <c r="C2" s="48" t="s">
-        <v>140</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-    </row>
-    <row r="3" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+    </row>
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="47" t="s">
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="45" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C12" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="45" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-    </row>
-    <row r="4" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="C4" s="48" t="s">
-        <v>143</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-    </row>
-    <row r="5" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="47" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="48" t="s">
-        <v>145</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-    </row>
-    <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="47" t="s">
-        <v>146</v>
-      </c>
-      <c r="C6" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A7" s="42"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" s="42"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A9" s="42"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A10" s="42"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A11" s="42"/>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A12" s="42"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A13" s="42"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A14" s="42"/>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A15" s="42"/>
-      <c r="B15" s="43"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A16" s="42"/>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A17" s="42"/>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A18" s="42"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
+    </row>
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="45" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" s="45" t="s">
+        <v>142</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1918,43 +2001,43 @@
           <x14:formula1>
             <xm:f>LookUp!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>C7:C17</xm:sqref>
+          <xm:sqref>C15:C22</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
+          <x14:formula1>
+            <xm:f>'Test Cases'!$A$2:$A$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I19</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
+          <x14:formula1>
+            <xm:f>LookUp!$E$2:$E$20</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H19</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000004000000}">
+          <x14:formula1>
+            <xm:f>'User Stories'!$A$2:$A$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>G15:G22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
           <x14:formula1>
             <xm:f>LookUp!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D17</xm:sqref>
+          <xm:sqref>D2:D22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000002000000}">
           <x14:formula1>
             <xm:f>LookUp!$D$2:$D$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E17</xm:sqref>
+          <xm:sqref>E2:E22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000003000000}">
           <x14:formula1>
             <xm:f>LookUp!$C$2:$C$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F17</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000004000000}">
-          <x14:formula1>
-            <xm:f>'User Stories'!$A$2:$A$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2 G7:G17</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
-          <x14:formula1>
-            <xm:f>'Test Cases'!$A$2:$A$18</xm:f>
-          </x14:formula1>
-          <xm:sqref>I2:I17</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
-          <x14:formula1>
-            <xm:f>LookUp!$E$2:$E$20</xm:f>
-          </x14:formula1>
-          <xm:sqref>H2:H17</xm:sqref>
+          <xm:sqref>F2:F22</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1965,201 +2048,201 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.3984375" customWidth="1"/>
-    <col min="3" max="3" width="19.1328125" customWidth="1"/>
-    <col min="4" max="4" width="21.59765625" customWidth="1"/>
-    <col min="5" max="5" width="20.73046875" customWidth="1"/>
-    <col min="6" max="6" width="22.1328125" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.65">
-      <c r="C1" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C2" s="37" t="s">
-        <v>90</v>
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="C1" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C2" s="43" t="s">
+        <v>85</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="38"/>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="44"/>
       <c r="D3" s="16" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="12"/>
       <c r="C4" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="12"/>
       <c r="C6" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="12"/>
       <c r="C7" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
       <c r="C8" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12"/>
       <c r="C9" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" s="12"/>
       <c r="C10" s="14" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" s="32"/>
+      <c r="F12" s="33"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="35"/>
+      <c r="F13" s="36"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="37"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="39"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="37"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="C16" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="37"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="39"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="E12" s="26"/>
-      <c r="F12" s="27"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B13" s="14" t="s">
+      <c r="C17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="40"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="42"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="30"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B14" s="14" t="s">
+      <c r="C18" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="33"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B15" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="33"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B16" s="14" t="s">
+      <c r="C19" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" s="31"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="33"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B17" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="36"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B18" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B19" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2177,256 +2260,256 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3984375" customWidth="1"/>
-    <col min="3" max="3" width="22.59765625" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.59765625" style="11" customWidth="1"/>
-    <col min="6" max="6" width="17.3984375" customWidth="1"/>
-    <col min="7" max="7" width="28.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="11" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -2436,17 +2519,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
-          <x14:formula1>
-            <xm:f>Anforderungen!$A$2:$A$17</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2:G18</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000001000000}">
           <x14:formula1>
             <xm:f>LookUp!$F$2:$F$4</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
+          <x14:formula1>
+            <xm:f>Anforderungen!$A$2:$A$23</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2457,242 +2540,242 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.73046875" customWidth="1"/>
-    <col min="3" max="3" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.1328125" customWidth="1"/>
-    <col min="6" max="6" width="15.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test Requirements begonnen zu definieren, Testumgebung definiert
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Elektrotechnik\6. Semester\Prozessortechnik\BPM-Detection\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6921A6DC-CE2F-4676-A028-22C148116EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F807ED91-47C4-42C5-B50D-9181D84E8D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="194">
   <si>
     <t>User Story ID</t>
   </si>
@@ -94,24 +94,6 @@
     <t>Log</t>
   </si>
   <si>
-    <t>TC_G5_1</t>
-  </si>
-  <si>
-    <t>TC_G5_2</t>
-  </si>
-  <si>
-    <t>TC_G5_3</t>
-  </si>
-  <si>
-    <t>TC_G5_4</t>
-  </si>
-  <si>
-    <t>TC_G5_5</t>
-  </si>
-  <si>
-    <t>TC_G5_6</t>
-  </si>
-  <si>
     <t>Inputs</t>
   </si>
   <si>
@@ -130,39 +112,6 @@
     <t>US_G5_5</t>
   </si>
   <si>
-    <t>TC_G5_7</t>
-  </si>
-  <si>
-    <t>TC_G5_8</t>
-  </si>
-  <si>
-    <t>TC_G5_9</t>
-  </si>
-  <si>
-    <t>TC_G5_10</t>
-  </si>
-  <si>
-    <t>TC_G5_11</t>
-  </si>
-  <si>
-    <t>TC_G5_12</t>
-  </si>
-  <si>
-    <t>TC_G5_13</t>
-  </si>
-  <si>
-    <t>TC_G5_14</t>
-  </si>
-  <si>
-    <t>TC_G5_15</t>
-  </si>
-  <si>
-    <t>TC_G5_16</t>
-  </si>
-  <si>
-    <t>TC_G5_17</t>
-  </si>
-  <si>
     <t>Anforderung Kategorie</t>
   </si>
   <si>
@@ -590,6 +539,216 @@
   </si>
   <si>
     <t>Die Entscheidung fällt auf Design 2 (FFT). Durch die Nutzung der CMSIS-DSP Library des Cortex-M7 lässt sich die Frequenzanalyse effizient umsetzen. Sie bietet eine deutlich höhere Robustheit gegenüber Rauschen im Vergleich zum einfachen Peak-Counting (Design 1). Design 3 fällt raus, da eine Autokorrelation zu viel Rechenleistung und Speicher braucht, was zu Problemen führen könnte.</t>
+  </si>
+  <si>
+    <t>TC_G1_1</t>
+  </si>
+  <si>
+    <t>TC_G1_2</t>
+  </si>
+  <si>
+    <t>TC_G1_3</t>
+  </si>
+  <si>
+    <t>TC_G1_4</t>
+  </si>
+  <si>
+    <t>TC_G1_5</t>
+  </si>
+  <si>
+    <t>TC_G1_6</t>
+  </si>
+  <si>
+    <t>TC_G1_7</t>
+  </si>
+  <si>
+    <t>TC_G1_8</t>
+  </si>
+  <si>
+    <t>TC_G1_9</t>
+  </si>
+  <si>
+    <t>TC_G1_10</t>
+  </si>
+  <si>
+    <t>TC_G1_11</t>
+  </si>
+  <si>
+    <t>TC_G1_12</t>
+  </si>
+  <si>
+    <t>TC_G1_13</t>
+  </si>
+  <si>
+    <t>TC_G1_14</t>
+  </si>
+  <si>
+    <t>TC_G1_15</t>
+  </si>
+  <si>
+    <t>TC_G1_16</t>
+  </si>
+  <si>
+    <t>TC_G1_17</t>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal 
+um +/-0.3 bpm von 
+Metadaten abweichen</t>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal um +/-0.3 BPM vom vom  Einspielgerät ermittelten Wert abweichen</t>
+  </si>
+  <si>
+    <t>Drumloop (4/4 Takt; Metadaten ermittelt)</t>
+  </si>
+  <si>
+    <t>Drumloop (4/4 Takt; 
+Metadaten nicht 
+ermittelt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des Musikstücks mit dem Einspielgerät </t>
+  </si>
+  <si>
+    <t>Musikstück (4/4 Takt; Metadaten ermittelt) mit anschließender Offbeat-Phase</t>
+  </si>
+  <si>
+    <t>Drumloop (4/4 Takt; 
+Metadaten ermittelt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
+  </si>
+  <si>
+    <t>Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Testumgebung:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Zum Testen wird ein professionelles Musikeinspielgerät, welches im Bereich der DJ-Technik zum Einsatz kommt, als Referenz und Musikquelle</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">eingesetzt. Beim Gerät handelt es sich um einen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pioneer XDJ-1000 Mk2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 
+Diesem liegt eine Software bei, mit welcher die Musik vorbereitet werden kann </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Rekordbox)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Die Software ermöglicht es unter anderem, die Musikstücke im Voraus zu analysieren und sogenannte </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Metadaten</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (BPM, Tonart,...) zu ermitteln.
+Das Einspielgerät ist darüberhinaus in der Lage, die BPM bei nicht analysierten Musikdaten selbstständig zu detektieren, sofern die Daten verwertbar sind.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Außerdem kann</t>
+    </r>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal um +/-0.3 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 2 Sekunden aktualisieren</t>
   </si>
 </sst>
 </file>
@@ -958,7 +1117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -983,9 +1142,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1054,37 +1210,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1368,57 +1539,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A1" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A2" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A3" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A4" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="33.5" x14ac:dyDescent="0.75">
-      <c r="A5" s="20" t="s">
+    <row r="1" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A1" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A2" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A3" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A4" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="21" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="34" thickBot="1" x14ac:dyDescent="0.8">
-      <c r="A6" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="23">
+    </row>
+    <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A5" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="22">
         <v>46133</v>
       </c>
     </row>
@@ -1431,18 +1602,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.26953125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.1796875" style="9" customWidth="1"/>
-    <col min="5" max="6" width="24" style="11" customWidth="1"/>
-    <col min="7" max="7" width="25.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.453125" style="6"/>
+    <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="9" customWidth="1"/>
+    <col min="5" max="6" width="24" style="10" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1456,154 +1627,154 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>47</v>
+        <v>122</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>30</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D3" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="7" t="s">
+      <c r="B6" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="87" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>134</v>
-      </c>
-      <c r="D6" s="26" t="s">
+      <c r="E7" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="E6" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="116" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D12" s="6"/>
     </row>
   </sheetData>
@@ -1639,345 +1810,345 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.453125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" style="32" customWidth="1"/>
-    <col min="4" max="4" width="11.453125" style="6"/>
-    <col min="5" max="5" width="13.26953125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" style="6"/>
-    <col min="7" max="8" width="23.453125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.26953125" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.453125" style="6"/>
+    <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="31" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="6"/>
+    <col min="7" max="8" width="23.42578125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="28" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="27" t="s">
+      <c r="H1" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>130</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>166</v>
+        <v>133</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>136</v>
-      </c>
-      <c r="C3" s="31" t="s">
-        <v>166</v>
+        <v>134</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="28" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>166</v>
+      <c r="C4" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>166</v>
+        <v>137</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="29" t="s">
-        <v>175</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>173</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>167</v>
+      <c r="C9" s="30" t="s">
+        <v>150</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>167</v>
+        <v>142</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>150</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>162</v>
+        <v>145</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>166</v>
+        <v>144</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>166</v>
+        <v>120</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="C13" s="31" t="s">
-        <v>166</v>
+        <v>147</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>166</v>
+        <v>148</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2037,228 +2208,228 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.453125" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" customWidth="1"/>
-    <col min="4" max="4" width="25.26953125" customWidth="1"/>
-    <col min="5" max="5" width="20.7265625" customWidth="1"/>
-    <col min="6" max="6" width="22.1796875" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.5">
-      <c r="C1" s="33" t="s">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="C1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C2" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="46"/>
+      <c r="D3" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="11"/>
+      <c r="C4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="11"/>
+      <c r="C6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="11"/>
+      <c r="C7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="11"/>
+      <c r="C8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="11"/>
+      <c r="C9" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="34"/>
+      <c r="F11" s="35"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="36" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="37"/>
+      <c r="F12" s="38"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="39"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="41"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="39"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="41"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="39"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="42"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="44"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C2" s="37" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="38"/>
-      <c r="D3" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B4" s="12"/>
-      <c r="C4" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B5" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B6" s="12"/>
-      <c r="C6" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B7" s="12"/>
-      <c r="C7" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="12"/>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="F8" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="12"/>
-      <c r="C9" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9" s="25" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D12" s="39" t="s">
-        <v>182</v>
-      </c>
-      <c r="E12" s="40"/>
-      <c r="F12" s="41"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D13" s="42"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D14" s="42"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="44"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="42"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="44"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B16" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D16" s="45"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="47"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B17" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B18" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2275,23 +2446,23 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.453125" customWidth="1"/>
-    <col min="3" max="3" width="22.54296875" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.54296875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" customWidth="1"/>
-    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>15</v>
@@ -2306,231 +2477,331 @@
         <v>16</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="48" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="47" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+    </row>
+    <row r="3" spans="1:7" s="48" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" s="47" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="47" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>190</v>
+      </c>
+      <c r="D3" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="E3" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+    </row>
+    <row r="4" spans="1:7" s="48" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="A4" s="47" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="47" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="49" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="E4" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+    </row>
+    <row r="5" spans="1:7" s="48" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="47" t="s">
+        <v>169</v>
+      </c>
+      <c r="B5" s="47" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="D5" s="47"/>
+      <c r="E5" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+    </row>
+    <row r="6" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+    </row>
+    <row r="7" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="47" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+    </row>
+    <row r="8" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="B8" s="47"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+    </row>
+    <row r="9" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="47"/>
+      <c r="G9" s="47"/>
+    </row>
+    <row r="10" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+    </row>
+    <row r="11" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="47" t="s">
+        <v>175</v>
+      </c>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+    </row>
+    <row r="12" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+    </row>
+    <row r="13" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
+    </row>
+    <row r="14" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="47" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+    </row>
+    <row r="15" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="47" t="s">
+        <v>179</v>
+      </c>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+    </row>
+    <row r="16" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="47" t="s">
+        <v>180</v>
+      </c>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+    </row>
+    <row r="17" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="47"/>
+      <c r="G17" s="47"/>
+    </row>
+    <row r="18" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="47"/>
+      <c r="G18" s="47"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="51" t="s">
+        <v>192</v>
+      </c>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="40"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="40"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="40"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B20:G28"/>
+  </mergeCells>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2556,242 +2827,242 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" customWidth="1"/>
-    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.1796875" customWidth="1"/>
-    <col min="6" max="6" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Req/Test Dokument formale Fehler korrigiert
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F807ED91-47C4-42C5-B50D-9181D84E8D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F968AA-3C37-471E-A952-CB51EC4B6643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="194">
   <si>
     <t>User Story ID</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Traceability Anforderungen</t>
   </si>
   <si>
-    <t>US_G5_2</t>
-  </si>
-  <si>
     <t>Text</t>
   </si>
   <si>
@@ -100,18 +97,6 @@
     <t>Anforderung ID</t>
   </si>
   <si>
-    <t>A_G5_1</t>
-  </si>
-  <si>
-    <t>A_G5_5</t>
-  </si>
-  <si>
-    <t>US_G5_4</t>
-  </si>
-  <si>
-    <t>US_G5_5</t>
-  </si>
-  <si>
     <t>Anforderung Kategorie</t>
   </si>
   <si>
@@ -406,9 +391,6 @@
     <t>Das System soll signalisieren, wenn keine zur Auswertung verwendbaren Daten am DSP anliegen (Break Part)</t>
   </si>
   <si>
-    <t>US_G5_6</t>
-  </si>
-  <si>
     <t>US_G1_1</t>
   </si>
   <si>
@@ -514,18 +496,9 @@
     <t>Das System muss auf der bereitgestellten Hardware (STM32F746G-DISCO) funktionieren ohne diese zu überlasten</t>
   </si>
   <si>
-    <t>US_G5_1\2\3\5\6</t>
-  </si>
-  <si>
     <t>Das System muss 4\4 Takte mit durchgehender Kickdrum erkennen können</t>
   </si>
   <si>
-    <t>US_G5_3\6</t>
-  </si>
-  <si>
-    <t>US_G5_1\3</t>
-  </si>
-  <si>
     <t>Echtzeitfähigkeit</t>
   </si>
   <si>
@@ -590,11 +563,6 @@
   </si>
   <si>
     <t>TC_G1_17</t>
-  </si>
-  <si>
-    <t>BPM-Wert darf maximal 
-um +/-0.3 bpm von 
-Metadaten abweichen</t>
   </si>
   <si>
     <t>BPM-Wert darf maximal um +/-0.3 BPM vom vom  Einspielgerät ermittelten Wert abweichen</t>
@@ -621,7 +589,13 @@
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
   </si>
   <si>
-    <t>Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern</t>
+    <t>BPM-Wert muss nach Übergang in Offbeat-Phase weiterhin angezeigt werden, Signalisierung von fehlender Messdaten muss erfolgen</t>
+  </si>
+  <si>
+    <t>Musikstück (4/4 Takt; Metadaten ermittelt)</t>
+  </si>
+  <si>
+    <t>Siehe TC_G1_1, wenn dies erfüllt ist, Signal pausieren</t>
   </si>
   <si>
     <r>
@@ -722,7 +696,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (BPM, Tonart,...) zu ermitteln.
-Das Einspielgerät ist darüberhinaus in der Lage, die BPM bei nicht analysierten Musikdaten selbstständig zu detektieren, sofern die Daten verwertbar sind.</t>
+Das Einspielgerät ist darüberhinaus in der Lage, die BPM bei nicht analysierten Musikdaten selbstständig zu detektieren, sofern die Daten verwertbar sind. Außerdem kann</t>
     </r>
     <r>
       <rPr>
@@ -733,8 +707,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
-</t>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -744,11 +717,38 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Außerdem kann</t>
+      <t>am Einspielgerät live die Geschwindigkeit des aktuellen Musikstücks verändert werden. Die Veränderung wird live angezeigt und ausgegeben</t>
     </r>
   </si>
   <si>
-    <t>BPM-Wert darf maximal um +/-0.3 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 2 Sekunden aktualisieren</t>
+    <t>BPM-Wert darf maximal 
+um +/-0.3 BPM von 
+Metadaten abweichen, LED muss im Takt blinken</t>
+  </si>
+  <si>
+    <t>US_G1_1\2\3\5\6</t>
+  </si>
+  <si>
+    <t>US_G1_3\6</t>
+  </si>
+  <si>
+    <t>US_G1_1\3</t>
+  </si>
+  <si>
+    <t>Energieversorgung erstmalig verbinden, System hochfahren lassen und erste Einspielung von Musik</t>
+  </si>
+  <si>
+    <t>System ist nach max. 60 Sekunden einsatzbereit und liest analoge Audiosignale über die Klinke-Schnittstelle ein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern (von 60 bis 180 BPM)
+</t>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal um +/-0.3 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 5 Sekunden aktualisieren</t>
+  </si>
+  <si>
+    <t>Sobald TC_G1_2 erfüllt ist und die Musik stoppt, muss der Wert für 10 Sekunden auf dem großen Display angezeigt werden und anschließend kleingedruckt am Bildschirmrand angezeigt werden, die Live Anzeige muss auf 0,0 zurückgesetzt werden</t>
   </si>
 </sst>
 </file>
@@ -1117,7 +1117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1198,6 +1198,24 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1222,9 +1240,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1243,20 +1258,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1539,55 +1542,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
       <c r="A1" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A2" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B2" s="20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A3" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A2" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A3" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
       <c r="A4" s="19" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
       <c r="A5" s="19" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A6" s="21" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B6" s="22">
         <v>46133</v>
@@ -1602,18 +1605,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.42578125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.44140625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" style="9" customWidth="1"/>
     <col min="5" max="6" width="24" style="10" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="6"/>
+    <col min="7" max="7" width="25.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.44140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1627,154 +1630,154 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="C2" s="25" t="s">
+      <c r="E4" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D2" s="25" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D12" s="6"/>
     </row>
   </sheetData>
@@ -1810,345 +1813,345 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="31" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="6"/>
-    <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="6"/>
-    <col min="7" max="8" width="23.42578125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="6"/>
+    <col min="1" max="1" width="14.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.44140625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" style="31" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" style="6"/>
+    <col min="5" max="5" width="13.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" style="6"/>
+    <col min="7" max="8" width="23.44140625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.33203125" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.44140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="D1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="E1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="F1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="G1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="H1" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="I1" s="26" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="C2" s="30" t="s">
+      <c r="B6" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>153</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="C14" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="C10" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>149</v>
-      </c>
       <c r="D14" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2162,12 +2165,6 @@
             <xm:f>LookUp!$A$2:$A$6</xm:f>
           </x14:formula1>
           <xm:sqref>C15:C22</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
-          <x14:formula1>
-            <xm:f>'Test Cases'!$A$2:$A$18</xm:f>
-          </x14:formula1>
-          <xm:sqref>I2:I19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
           <x14:formula1>
@@ -2199,6 +2196,12 @@
           </x14:formula1>
           <xm:sqref>F2:F22</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
+          <x14:formula1>
+            <xm:f>'Test Cases'!$A$3:$A$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I19</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -2208,228 +2211,228 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="C1" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C2" s="45" t="s">
-        <v>67</v>
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
+      <c r="C1" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C2" s="50" t="s">
+        <v>62</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="46"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="51"/>
       <c r="D3" s="15" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="11"/>
       <c r="C4" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="12" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6" s="11"/>
       <c r="C6" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" s="11"/>
       <c r="C7" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" s="11"/>
       <c r="C8" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" s="11"/>
       <c r="C9" s="13" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="D9" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="40"/>
+      <c r="F11" s="41"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="E12" s="43"/>
+      <c r="F12" s="44"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="45"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="46"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="45"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="46"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="45"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="46"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="47"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="35"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>165</v>
-      </c>
-      <c r="E12" s="37"/>
-      <c r="F12" s="38"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" s="39"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="41"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="39"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="41"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="42"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="44"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2447,355 +2450,381 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" customWidth="1"/>
+    <col min="3" max="3" width="22.5546875" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="28.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="G1" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="48" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="33" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>190</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="32"/>
+      <c r="G2" s="52" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="33" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="33" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="32" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="E4" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="33" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="33" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>178</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>181</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="33" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="32" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+    </row>
+    <row r="9" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+    </row>
+    <row r="10" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+    </row>
+    <row r="11" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="49" t="s">
-        <v>185</v>
-      </c>
-      <c r="C2" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="E2" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-    </row>
-    <row r="3" spans="1:7" s="48" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+    </row>
+    <row r="12" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="B3" s="47" t="s">
-        <v>186</v>
-      </c>
-      <c r="C3" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="D3" s="47" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+    </row>
+    <row r="13" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+    </row>
+    <row r="14" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+    </row>
+    <row r="15" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="32" t="s">
+        <v>170</v>
+      </c>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+    </row>
+    <row r="16" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+    </row>
+    <row r="17" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+    </row>
+    <row r="18" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="E3" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-    </row>
-    <row r="4" spans="1:7" s="48" customFormat="1" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" s="47" t="s">
-        <v>168</v>
-      </c>
-      <c r="B4" s="47" t="s">
-        <v>189</v>
-      </c>
-      <c r="C4" s="49" t="s">
-        <v>191</v>
-      </c>
-      <c r="D4" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="E4" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-    </row>
-    <row r="5" spans="1:7" s="48" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
-        <v>169</v>
-      </c>
-      <c r="B5" s="47" t="s">
-        <v>188</v>
-      </c>
-      <c r="C5" s="47" t="s">
-        <v>187</v>
-      </c>
-      <c r="D5" s="47"/>
-      <c r="E5" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-    </row>
-    <row r="6" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="47" t="s">
-        <v>170</v>
-      </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-    </row>
-    <row r="7" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
-        <v>171</v>
-      </c>
-      <c r="B7" s="47"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-    </row>
-    <row r="8" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="47" t="s">
-        <v>172</v>
-      </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-    </row>
-    <row r="9" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="47" t="s">
-        <v>173</v>
-      </c>
-      <c r="B9" s="47"/>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="47"/>
-      <c r="G9" s="47"/>
-    </row>
-    <row r="10" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="47" t="s">
-        <v>174</v>
-      </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-    </row>
-    <row r="11" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="47" t="s">
-        <v>175</v>
-      </c>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-    </row>
-    <row r="12" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
-        <v>176</v>
-      </c>
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-    </row>
-    <row r="13" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="B13" s="47"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-    </row>
-    <row r="14" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-    </row>
-    <row r="15" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
-        <v>179</v>
-      </c>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" s="47"/>
-      <c r="G15" s="47"/>
-    </row>
-    <row r="16" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="47" t="s">
-        <v>180</v>
-      </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" s="47"/>
-      <c r="G16" s="47"/>
-    </row>
-    <row r="17" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
-        <v>181</v>
-      </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" s="47"/>
-      <c r="G17" s="47"/>
-    </row>
-    <row r="18" spans="1:7" s="48" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B18" s="47"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" s="47"/>
-      <c r="G18" s="47"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="51" t="s">
-        <v>192</v>
-      </c>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B25" s="40"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2803,6 +2832,7 @@
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -2810,13 +2840,13 @@
           <x14:formula1>
             <xm:f>LookUp!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E18</xm:sqref>
+          <xm:sqref>E8:E18 E2:E7</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
             <xm:f>Anforderungen!$A$2:$A$23</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G18</xm:sqref>
+          <xm:sqref>G8:G18 G2:G7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2827,242 +2857,242 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.140625" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.109375" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test Protokolle 1-3 hinzugefügt
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD156868-C857-4792-BA60-486E8C1A4D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0861673B-F9D7-4CC0-A7E5-B916253FE7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -540,9 +540,6 @@
   <si>
     <t>Drumloop (4/4 Takt; 
 Metadaten ermittelt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
   </si>
   <si>
     <t>BPM-Wert muss nach Übergang in Offbeat-Phase weiterhin angezeigt werden, Signalisierung von fehlender Messdaten muss erfolgen</t>
@@ -686,9 +683,6 @@
     <t>US_G1_1\3</t>
   </si>
   <si>
-    <t>Energieversorgung erstmalig verbinden, System hochfahren lassen und erste Einspielung von Musik</t>
-  </si>
-  <si>
     <t>System ist nach max. 60 Sekunden einsatzbereit und liest analoge Audiosignale über die Klinke-Schnittstelle ein</t>
   </si>
   <si>
@@ -697,11 +691,6 @@
   </si>
   <si>
     <t>Sobald TC_G1_2 erfüllt ist und die Musik stoppt, muss der Wert für 10 Sekunden auf dem großen Display angezeigt werden und anschließend kleingedruckt am Bildschirmrand angezeigt werden, die Live Anzeige muss auf 0,0 zurückgesetzt werden</t>
-  </si>
-  <si>
-    <t>BPM-Wert darf maximal 
-um +/- 2 BPM von 
-Metadaten abweichen, LED muss im Takt blinken</t>
   </si>
   <si>
     <t>BPM-Wert darf maximal um +/- 2 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 5 Sekunden aktualisieren</t>
@@ -722,6 +711,19 @@
     <t>A_G1_10
 A_G1_11
 A_G1_12</t>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal 
+um +/- 2 BPM von 
+Metadaten abweichen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energieversorgung erstmalig verbinden, System hochfahren lassen und erste Einspielung von Musik
+</t>
   </si>
 </sst>
 </file>
@@ -1183,6 +1185,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1230,12 +1238,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1518,13 +1520,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A1" s="17" t="s">
         <v>89</v>
       </c>
@@ -1532,7 +1534,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="2" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A2" s="19" t="s">
         <v>94</v>
       </c>
@@ -1540,7 +1542,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A3" s="19" t="s">
         <v>95</v>
       </c>
@@ -1548,7 +1550,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A4" s="19" t="s">
         <v>90</v>
       </c>
@@ -1556,7 +1558,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A5" s="19" t="s">
         <v>92</v>
       </c>
@@ -1564,7 +1566,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="21" t="s">
         <v>91</v>
       </c>
@@ -1581,18 +1583,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.44140625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.109375" style="9" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="9" customWidth="1"/>
     <col min="5" max="6" width="24" style="10" customWidth="1"/>
-    <col min="7" max="7" width="25.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.44140625" style="6"/>
+    <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1615,7 +1617,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>116</v>
       </c>
@@ -1638,7 +1640,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>117</v>
       </c>
@@ -1661,7 +1663,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>118</v>
       </c>
@@ -1684,7 +1686,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>119</v>
       </c>
@@ -1707,7 +1709,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>120</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>132</v>
       </c>
@@ -1753,7 +1755,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D12" s="6"/>
     </row>
   </sheetData>
@@ -1789,20 +1791,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.44140625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="31" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" style="6"/>
-    <col min="5" max="5" width="13.33203125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" style="6"/>
-    <col min="7" max="8" width="23.44140625" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.33203125" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="11.44140625" style="6"/>
+    <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="31" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="6"/>
+    <col min="7" max="8" width="23.42578125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>17</v>
       </c>
@@ -1831,7 +1833,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>127</v>
       </c>
@@ -1851,10 +1853,10 @@
         <v>25</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>128</v>
       </c>
@@ -1877,7 +1879,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>130</v>
       </c>
@@ -1897,10 +1899,10 @@
         <v>25</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>131</v>
       </c>
@@ -1923,7 +1925,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>133</v>
       </c>
@@ -1943,10 +1945,10 @@
         <v>25</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>134</v>
       </c>
@@ -1966,10 +1968,10 @@
         <v>25</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>129</v>
       </c>
@@ -1989,10 +1991,10 @@
         <v>25</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>135</v>
       </c>
@@ -2015,7 +2017,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>136</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>139</v>
       </c>
@@ -2061,7 +2063,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>140</v>
       </c>
@@ -2084,7 +2086,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>148</v>
       </c>
@@ -2107,7 +2109,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>149</v>
       </c>
@@ -2187,25 +2189,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.44140625" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" customWidth="1"/>
-    <col min="4" max="4" width="25.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="C1" s="38" t="s">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="C1" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C2" s="50" t="s">
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C2" s="52" t="s">
         <v>62</v>
       </c>
       <c r="D2" s="14" t="s">
@@ -2218,8 +2220,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="51"/>
+    <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="53"/>
       <c r="D3" s="15" t="s">
         <v>153</v>
       </c>
@@ -2230,7 +2232,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="11"/>
       <c r="C4" s="2" t="s">
         <v>74</v>
@@ -2245,7 +2247,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -2262,7 +2264,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="11"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
@@ -2277,7 +2279,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="11"/>
       <c r="C7" s="2" t="s">
         <v>57</v>
@@ -2292,7 +2294,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -2307,7 +2309,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="11"/>
       <c r="C9" s="13" t="s">
         <v>152</v>
@@ -2322,7 +2324,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>65</v>
       </c>
@@ -2332,70 +2334,70 @@
       <c r="C11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="40"/>
-      <c r="F11" s="41"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E11" s="42"/>
+      <c r="F11" s="43"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" s="13" t="s">
         <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="42" t="s">
+      <c r="D12" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E12" s="45"/>
+      <c r="F12" s="46"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="13" t="s">
         <v>68</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="45"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="46"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D13" s="47"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="48"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>69</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="45"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="46"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D14" s="47"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="48"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="13" t="s">
         <v>70</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="45"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="46"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D15" s="47"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="48"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="47"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
         <v>72</v>
       </c>
@@ -2403,7 +2405,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>73</v>
       </c>
@@ -2426,18 +2428,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="10" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.44140625" style="53" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.42578125" style="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -2459,11 +2461,11 @@
       <c r="G1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="36" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="33" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="33" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="32" t="s">
         <v>157</v>
       </c>
@@ -2471,10 +2473,10 @@
         <v>162</v>
       </c>
       <c r="C2" s="32" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E2" s="35" t="s">
         <v>25</v>
@@ -2484,10 +2486,10 @@
         <v>127</v>
       </c>
       <c r="H2" s="32" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="33" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="33" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>158</v>
       </c>
@@ -2495,10 +2497,10 @@
         <v>162</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E3" s="35" t="s">
         <v>25</v>
@@ -2508,10 +2510,10 @@
         <v>128</v>
       </c>
       <c r="H3" s="32" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="33" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="33" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
         <v>159</v>
       </c>
@@ -2519,10 +2521,10 @@
         <v>165</v>
       </c>
       <c r="C4" s="34" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="32" t="s">
         <v>176</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>179</v>
       </c>
       <c r="E4" s="35" t="s">
         <v>25</v>
@@ -2535,7 +2537,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="33" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" s="33" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
         <v>160</v>
       </c>
@@ -2546,7 +2548,7 @@
         <v>163</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E5" s="35" t="s">
         <v>25</v>
@@ -2556,21 +2558,21 @@
         <v>139</v>
       </c>
       <c r="H5" s="32" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="33" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="33" customFormat="1" ht="195" x14ac:dyDescent="0.25">
       <c r="A6" s="32" t="s">
         <v>161</v>
       </c>
       <c r="B6" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>169</v>
-      </c>
       <c r="D6" s="32" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E6" s="35" t="s">
         <v>25</v>
@@ -2583,7 +2585,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7"/>
       <c r="B7"/>
       <c r="C7"/>
@@ -2593,99 +2595,99 @@
       <c r="G7"/>
       <c r="H7" s="34"/>
     </row>
-    <row r="8" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
-      <c r="B8" s="36" t="s">
-        <v>170</v>
-      </c>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
+      <c r="B8" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
       <c r="H8" s="34"/>
     </row>
-    <row r="9" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
       <c r="H9" s="34"/>
     </row>
-    <row r="10" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
       <c r="H10" s="34"/>
     </row>
-    <row r="11" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
       <c r="H11" s="34"/>
     </row>
-    <row r="12" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="37"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
       <c r="H12" s="34"/>
     </row>
-    <row r="13" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
       <c r="H13" s="34"/>
     </row>
-    <row r="14" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
       <c r="H14" s="34"/>
     </row>
-    <row r="15" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
       <c r="H15" s="34"/>
     </row>
-    <row r="16" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37"/>
+      <c r="B16" s="39"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
       <c r="H16" s="34"/>
     </row>
-    <row r="17" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
       <c r="B17"/>
       <c r="C17"/>
@@ -2695,7 +2697,7 @@
       <c r="G17"/>
       <c r="H17" s="34"/>
     </row>
-    <row r="18" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18"/>
@@ -2703,7 +2705,7 @@
       <c r="E18" s="10"/>
       <c r="F18"/>
       <c r="G18"/>
-      <c r="H18" s="53"/>
+      <c r="H18" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2736,17 +2738,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.109375" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -2766,7 +2768,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
@@ -2786,7 +2788,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -2806,7 +2808,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -2826,7 +2828,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>29</v>
       </c>
@@ -2837,7 +2839,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -2848,7 +2850,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2857,7 +2859,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2866,7 +2868,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -2875,7 +2877,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2884,7 +2886,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2893,7 +2895,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2902,7 +2904,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2911,7 +2913,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2920,7 +2922,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2929,7 +2931,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2938,7 +2940,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -2947,7 +2949,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -2956,7 +2958,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2965,7 +2967,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>

</xml_diff>

<commit_message>
Failed Commit korrigiert, jetzt Test Protokolle 1-3 online
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://primion-my.sharepoint.com/personal/david_roesch_primion_eu/Documents/Studium/Semester 6/Prozessortechnik/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0861673B-F9D7-4CC0-A7E5-B916253FE7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{DD156868-C857-4792-BA60-486E8C1A4D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEB64F6A-29FB-4BA4-B450-F4EC330D69B4}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="186">
   <si>
     <t>User Story ID</t>
   </si>
@@ -331,9 +331,6 @@
     <t>Projektthema</t>
   </si>
   <si>
-    <t>z.B. 1.0</t>
-  </si>
-  <si>
     <t>Gruppe 1</t>
   </si>
   <si>
@@ -368,9 +365,6 @@
   </si>
   <si>
     <t>Das System muss ein analoges Audiosignal über einen Line-In (z. B. Klinke) empfangen und mittels ADC für den DSP digitalisieren.</t>
-  </si>
-  <si>
-    <t>Felix Maunz</t>
   </si>
   <si>
     <t>Als Entwickler von Audio-Hardware, möchte ich die BPM-Berechnung direkt auf einem integrierten DSP durchführen, damit ich eine extrem geringe Latenz erreiche und die Haupt-CPU des Mikrocontrollers für andere Aufgaben (wie das Display-Rendering) entlaste.</t>
@@ -542,13 +536,75 @@
 Metadaten ermittelt)</t>
   </si>
   <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
+  </si>
+  <si>
     <t>BPM-Wert muss nach Übergang in Offbeat-Phase weiterhin angezeigt werden, Signalisierung von fehlender Messdaten muss erfolgen</t>
   </si>
   <si>
     <t>Musikstück (4/4 Takt; Metadaten ermittelt)</t>
   </si>
   <si>
-    <t>Siehe TC_G1_1, wenn dies erfüllt ist, Signal pausieren</t>
+    <t>US_G1_1\2\3\5\6</t>
+  </si>
+  <si>
+    <t>US_G1_3\6</t>
+  </si>
+  <si>
+    <t>US_G1_1\3</t>
+  </si>
+  <si>
+    <t>System ist nach max. 60 Sekunden einsatzbereit und liest analoge Audiosignale über die Klinke-Schnittstelle ein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern (von 60 bis 180 BPM)
+</t>
+  </si>
+  <si>
+    <t>Sobald TC_G1_2 erfüllt ist und die Musik stoppt, muss der Wert für 10 Sekunden auf dem großen Display angezeigt werden und anschließend kleingedruckt am Bildschirmrand angezeigt werden, die Live Anzeige muss auf 0,0 zurückgesetzt werden</t>
+  </si>
+  <si>
+    <t>BPM-Wert darf maximal um +/- 2 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 5 Sekunden aktualisieren</t>
+  </si>
+  <si>
+    <t>A_G1_2
+A_G1_4
+A_G1_5</t>
+  </si>
+  <si>
+    <t>A_G1_1
+A_G1_2
+A_G1_6
+A_G1_8
+A_G1_9</t>
+  </si>
+  <si>
+    <t>A_G1_10
+A_G1_11
+A_G1_12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BPM-Wert darf maximal 
+um +/- 2 BPM von 
+Metadaten abweichen
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energieversorgung erstmalig verbinden, System hochfahren lassen und erste Einspielung von Musik
+</t>
+  </si>
+  <si>
+    <t>Siehe TC_G1_2, wenn dies erfüllt ist, Signal pausieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> LED muss im Takt blinken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät 
+</t>
+  </si>
+  <si>
+    <t>TC_G1_6</t>
   </si>
   <si>
     <r>
@@ -649,81 +705,14 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (BPM, Tonart,...) zu ermitteln.
-Das Einspielgerät ist darüberhinaus in der Lage, die BPM bei nicht analysierten Musikdaten selbstständig zu detektieren, sofern die Daten verwertbar sind. Außerdem kann</t>
+Am Einspielgerät kann die Geschwindigkeit des aktuellen Musikstücks verändert werden. Die Veränderung wird live angezeigt und ausgegeben</t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>am Einspielgerät live die Geschwindigkeit des aktuellen Musikstücks verändert werden. Die Veränderung wird live angezeigt und ausgegeben</t>
-    </r>
-  </si>
-  <si>
-    <t>US_G1_1\2\3\5\6</t>
-  </si>
-  <si>
-    <t>US_G1_3\6</t>
-  </si>
-  <si>
-    <t>US_G1_1\3</t>
-  </si>
-  <si>
-    <t>System ist nach max. 60 Sekunden einsatzbereit und liest analoge Audiosignale über die Klinke-Schnittstelle ein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern (von 60 bis 180 BPM)
-</t>
-  </si>
-  <si>
-    <t>Sobald TC_G1_2 erfüllt ist und die Musik stoppt, muss der Wert für 10 Sekunden auf dem großen Display angezeigt werden und anschließend kleingedruckt am Bildschirmrand angezeigt werden, die Live Anzeige muss auf 0,0 zurückgesetzt werden</t>
-  </si>
-  <si>
-    <t>BPM-Wert darf maximal um +/- 2 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 5 Sekunden aktualisieren</t>
-  </si>
-  <si>
-    <t>A_G1_2
-A_G1_4
-A_G1_5</t>
-  </si>
-  <si>
-    <t>A_G1_1
-A_G1_2
-A_G1_6
-A_G1_8
-A_G1_9</t>
-  </si>
-  <si>
-    <t>A_G1_10
-A_G1_11
-A_G1_12</t>
-  </si>
-  <si>
-    <t>BPM-Wert darf maximal 
-um +/- 2 BPM von 
-Metadaten abweichen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät 
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energieversorgung erstmalig verbinden, System hochfahren lassen und erste Einspielung von Musik
-</t>
+  </si>
+  <si>
+    <t>David Rösch</t>
+  </si>
+  <si>
+    <t>3.2</t>
   </si>
 </sst>
 </file>
@@ -821,7 +810,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -902,17 +891,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -922,7 +900,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -934,48 +914,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -1092,7 +1030,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1115,9 +1053,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1133,20 +1068,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1158,12 +1090,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1191,6 +1117,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1218,26 +1156,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1254,6 +1183,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1527,51 +1460,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A3" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A3" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>98</v>
-      </c>
-    </row>
     <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>109</v>
+      <c r="B4" s="19" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="20" t="s">
-        <v>96</v>
+      <c r="B5" s="50" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="22">
-        <v>46133</v>
+      <c r="B6" s="21">
+        <v>46183</v>
       </c>
     </row>
   </sheetData>
@@ -1587,9 +1520,9 @@
   <cols>
     <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
     <col min="2" max="2" width="20.140625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42.42578125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" style="9" customWidth="1"/>
-    <col min="5" max="6" width="24" style="10" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" style="30" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="30" customWidth="1"/>
+    <col min="5" max="6" width="24" style="9" customWidth="1"/>
     <col min="7" max="7" width="25.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="11.42578125" style="6"/>
   </cols>
@@ -1601,10 +1534,10 @@
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="36" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
@@ -1619,144 +1552,144 @@
     </row>
     <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>121</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>145</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D12" s="6"/>
+      <c r="D12" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1794,8 +1727,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="31" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" style="30" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="27" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" style="6"/>
     <col min="5" max="5" width="13.28515625" style="6" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="6"/>
@@ -1805,43 +1738,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="24" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>143</v>
+        <v>125</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>30</v>
@@ -1853,18 +1786,18 @@
         <v>25</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>143</v>
+        <v>126</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>25</v>
@@ -1876,18 +1809,18 @@
         <v>25</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>143</v>
+        <v>128</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>25</v>
@@ -1899,18 +1832,18 @@
         <v>25</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>143</v>
+        <v>129</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>25</v>
@@ -1922,18 +1855,18 @@
         <v>25</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>143</v>
+        <v>131</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>25</v>
@@ -1945,18 +1878,18 @@
         <v>25</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>143</v>
+        <v>132</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>25</v>
@@ -1968,18 +1901,18 @@
         <v>25</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>143</v>
+        <v>127</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>25</v>
@@ -1991,18 +1924,18 @@
         <v>25</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>144</v>
+        <v>133</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>142</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>25</v>
@@ -2014,18 +1947,18 @@
         <v>25</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>137</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>144</v>
+        <v>134</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>142</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>25</v>
@@ -2037,18 +1970,18 @@
         <v>25</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>143</v>
+        <v>137</v>
+      </c>
+      <c r="B11" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>25</v>
@@ -2060,18 +1993,18 @@
         <v>25</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>143</v>
+        <v>138</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>25</v>
@@ -2083,19 +2016,19 @@
         <v>25</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="B13" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="C13" s="30" t="s">
-        <v>143</v>
-      </c>
       <c r="D13" s="7" t="s">
         <v>25</v>
       </c>
@@ -2106,18 +2039,18 @@
         <v>25</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>143</v>
+        <v>147</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>25</v>
@@ -2129,7 +2062,7 @@
         <v>25</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2176,7 +2109,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
           <x14:formula1>
-            <xm:f>'Test Cases'!$A$3:$A$6</xm:f>
+            <xm:f>'Test Cases'!$A$3:$A$7</xm:f>
           </x14:formula1>
           <xm:sqref>I2:I19</xm:sqref>
         </x14:dataValidation>
@@ -2207,120 +2140,120 @@
       <c r="F1" s="40"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="13" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="53"/>
-      <c r="D3" s="15" t="s">
+      <c r="C3" s="48"/>
+      <c r="D3" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F3" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>155</v>
-      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="11"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="22" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="22" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="11"/>
+      <c r="B6" s="10"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="22" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="11"/>
+      <c r="B7" s="10"/>
       <c r="C7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="22" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="11"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="22" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="11"/>
-      <c r="C9" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="D9" s="24" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="22" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2328,7 +2261,7 @@
       <c r="A11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="12" t="s">
         <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -2340,29 +2273,29 @@
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="13" t="s">
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="12" t="s">
         <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E12" s="45"/>
-      <c r="F12" s="46"/>
+      <c r="F12" s="45"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="12" t="s">
         <v>68</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="48"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
@@ -2371,54 +2304,60 @@
       <c r="C14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="47"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="48"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>70</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="47"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="48"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="12" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="51"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="13" t="s">
+      <c r="D16" s="46"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="12" t="s">
         <v>72</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="46"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>75</v>
       </c>
+      <c r="D18" s="46"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F16"/>
     <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D12:F18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -2427,16 +2366,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.42578125" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="9" customWidth="1"/>
     <col min="6" max="6" width="17.42578125" customWidth="1"/>
     <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.42578125" style="37" customWidth="1"/>
+    <col min="8" max="8" width="28.42578125" style="33" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2461,163 +2400,175 @@
       <c r="G1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="H1" s="32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="33" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+    <row r="2" spans="1:8" s="29" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="29" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="29" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+      <c r="A4" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B4" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="29" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="1:8" s="29" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C6" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="29" customFormat="1" ht="195" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="32" t="s">
-        <v>173</v>
-      </c>
-      <c r="E2" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32" t="s">
-        <v>127</v>
-      </c>
-      <c r="H2" s="32" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="33" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
-        <v>158</v>
-      </c>
-      <c r="B3" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>181</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>180</v>
-      </c>
-      <c r="E3" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32" t="s">
-        <v>128</v>
-      </c>
-      <c r="H3" s="32" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="33" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>174</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32" t="s">
-        <v>130</v>
-      </c>
-      <c r="H4" s="32" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="33" customFormat="1" ht="105" x14ac:dyDescent="0.25">
-      <c r="A5" s="32" t="s">
-        <v>160</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>164</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="D5" s="32" t="s">
+      <c r="B7" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="E5" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="H5" s="32" t="s">
+      <c r="C7" s="28" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" s="33" customFormat="1" ht="195" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>168</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>175</v>
-      </c>
-      <c r="E6" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32" t="s">
-        <v>149</v>
-      </c>
-      <c r="H6" s="32" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7"/>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7" s="10"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7" s="34"/>
-    </row>
-    <row r="8" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
-      <c r="B8" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="34"/>
-    </row>
-    <row r="9" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8" s="9"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8" s="30"/>
+    </row>
+    <row r="9" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
-      <c r="B9" s="39"/>
+      <c r="B9" s="38" t="s">
+        <v>183</v>
+      </c>
       <c r="C9" s="39"/>
       <c r="D9" s="39"/>
       <c r="E9" s="39"/>
       <c r="F9" s="39"/>
       <c r="G9" s="39"/>
-      <c r="H9" s="34"/>
-    </row>
-    <row r="10" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="30"/>
+    </row>
+    <row r="10" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
       <c r="B10" s="39"/>
       <c r="C10" s="39"/>
@@ -2625,9 +2576,9 @@
       <c r="E10" s="39"/>
       <c r="F10" s="39"/>
       <c r="G10" s="39"/>
-      <c r="H10" s="34"/>
-    </row>
-    <row r="11" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H10" s="30"/>
+    </row>
+    <row r="11" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
       <c r="B11" s="39"/>
       <c r="C11" s="39"/>
@@ -2635,9 +2586,9 @@
       <c r="E11" s="39"/>
       <c r="F11" s="39"/>
       <c r="G11" s="39"/>
-      <c r="H11" s="34"/>
-    </row>
-    <row r="12" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="30"/>
+    </row>
+    <row r="12" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
       <c r="B12" s="39"/>
       <c r="C12" s="39"/>
@@ -2645,9 +2596,9 @@
       <c r="E12" s="39"/>
       <c r="F12" s="39"/>
       <c r="G12" s="39"/>
-      <c r="H12" s="34"/>
-    </row>
-    <row r="13" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H12" s="30"/>
+    </row>
+    <row r="13" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
@@ -2655,9 +2606,9 @@
       <c r="E13" s="39"/>
       <c r="F13" s="39"/>
       <c r="G13" s="39"/>
-      <c r="H13" s="34"/>
-    </row>
-    <row r="14" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H13" s="30"/>
+    </row>
+    <row r="14" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
       <c r="B14" s="39"/>
       <c r="C14" s="39"/>
@@ -2665,9 +2616,9 @@
       <c r="E14" s="39"/>
       <c r="F14" s="39"/>
       <c r="G14" s="39"/>
-      <c r="H14" s="34"/>
-    </row>
-    <row r="15" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H14" s="30"/>
+    </row>
+    <row r="15" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
       <c r="B15" s="39"/>
       <c r="C15" s="39"/>
@@ -2675,9 +2626,9 @@
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="39"/>
-      <c r="H15" s="34"/>
-    </row>
-    <row r="16" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H15" s="30"/>
+    </row>
+    <row r="16" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
       <c r="B16" s="39"/>
       <c r="C16" s="39"/>
@@ -2685,35 +2636,45 @@
       <c r="E16" s="39"/>
       <c r="F16" s="39"/>
       <c r="G16" s="39"/>
-      <c r="H16" s="34"/>
-    </row>
-    <row r="17" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H16" s="30"/>
+    </row>
+    <row r="17" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
-      <c r="B17"/>
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17" s="10"/>
-      <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17" s="34"/>
-    </row>
-    <row r="18" spans="1:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="39"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="30"/>
+    </row>
+    <row r="18" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18"/>
       <c r="G18"/>
-      <c r="H18" s="37"/>
+      <c r="H18" s="30"/>
+    </row>
+    <row r="19" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19"/>
+      <c r="B19"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19" s="9"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B8:G16"/>
+    <mergeCell ref="B9:G17"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -2721,13 +2682,13 @@
           <x14:formula1>
             <xm:f>LookUp!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E6</xm:sqref>
+          <xm:sqref>E2:E7</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
             <xm:f>Anforderungen!$A$2:$A$23</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G6</xm:sqref>
+          <xm:sqref>G2:G7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2764,7 +2725,7 @@
       <c r="E1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="15" t="s">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test Protokoll 4 hinzugefügt
</commit_message>
<xml_diff>
--- a/doc/Stories_Req_Design_Test_Template.xlsx
+++ b/doc/Stories_Req_Design_Test_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://primion-my.sharepoint.com/personal/david_roesch_primion_eu/Documents/Studium/Semester 6/Prozessortechnik/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david.roesch\Documents\Github\BPM-Detection\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{DD156868-C857-4792-BA60-486E8C1A4D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEB64F6A-29FB-4BA4-B450-F4EC330D69B4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F79781-C4C9-4EDE-AA20-F959AFE3AF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="164">
   <si>
     <t>User Story ID</t>
   </si>
@@ -382,9 +382,6 @@
     <t>Der DSP-Algorithmus muss den Grundtakt (Beat) aus dem digitalen Signal nahezu in Echtzeit extrahieren(maximale Latenz 5 Sekunden).</t>
   </si>
   <si>
-    <t>Das System soll signalisieren, wenn keine zur Auswertung verwendbaren Daten am DSP anliegen (Break Part)</t>
-  </si>
-  <si>
     <t>US_G1_1</t>
   </si>
   <si>
@@ -412,12 +409,6 @@
     <t>Als Schlagzeuger in einer Band, die mit vorproduzierten Backing-Tracks arbeitet, möchte ich das aktuelle Tempo des analogen Mixers in Echtzeit auf einem Display sehen, damit ich erkenne, ob wir aus dem Takt geraten, ohne auf ein komplexes Laptop-Setup angewiesen zu sein.</t>
   </si>
   <si>
-    <t>Der DJ (Getaktete Effekte)</t>
-  </si>
-  <si>
-    <t>Als Vinyl-DJ, der rein analoge Plattenspieler nutzt um House und Techno aufzulegen, möchte ich eine präzise digitale BPM-Anzeige für mein analoges Audiosignal haben, damit ich meine externen Effektgeräte an die BPM angleichen kann. Gerade in den Breakparts ohne Drums ist der Einsatz von Effekten ein wichtiger Bestandteil des Mixings</t>
-  </si>
-  <si>
     <t>A_G1_1</t>
   </si>
   <si>
@@ -433,9 +424,6 @@
     <t>A_G1_4</t>
   </si>
   <si>
-    <t>US_G1_6</t>
-  </si>
-  <si>
     <t>A_G1_5</t>
   </si>
   <si>
@@ -451,42 +439,18 @@
     <t>Das System muss innerhalb von 60 Sekunden nach Start der Energieversorgung selbstständig und ohne zusätzliche Betätigungen durch den User "ready to use" sein</t>
   </si>
   <si>
-    <t>Das System muss zwischen keinen Daten (kein Audiosignal) und keinen verwertbaren Daten (keine getaktete Musik, andere Audiosignale) unterscheiden</t>
-  </si>
-  <si>
-    <t>A_G1_10</t>
-  </si>
-  <si>
-    <t>A_G1_11</t>
-  </si>
-  <si>
-    <t>Das System soll den letzten ausgewerteten BPM-Wert solange anzeigen bis entweder eine neue Auswertung erfolgt ist oder das Audiosignal für mehr als 10 Sekunden unterbrochen wurde</t>
-  </si>
-  <si>
-    <t>Das System soll , wenn das Audiosignal für mehr als 10 Sekunden unterbrochen wurde, den Live Wert auf 0 BPM setzen und den letzten gemessenen Wert in einer Ecke des Displays kleingedruckt anzeigen</t>
-  </si>
-  <si>
     <t>Funktional</t>
   </si>
   <si>
     <t>Nicht-Funktional</t>
   </si>
   <si>
-    <t xml:space="preserve">Das System muss bei anliegenden Audiodaten, die nicht auswertbar sind den letzten erfassten Wert weiterhin auf dem Display anzeigen, aber visuell darauf hinweisen, dass dieser Wert nicht mehr live gemessen wurde </t>
-  </si>
-  <si>
     <t>Das System muss den gemessenen BPM-Wert auf 1/10 BPM genau anzeigen</t>
   </si>
   <si>
     <t>Das System muss einen Tempobereich von mindestens 60 bis 180 BPM (Beats Per Minute) abdecken.</t>
   </si>
   <si>
-    <t>A_G1_12</t>
-  </si>
-  <si>
-    <t>A_G1_13</t>
-  </si>
-  <si>
     <t>Das System muss auf der bereitgestellten Hardware (STM32F746G-DISCO) funktionieren ohne diese zu überlasten</t>
   </si>
   <si>
@@ -520,16 +484,7 @@
     <t>TC_G1_4</t>
   </si>
   <si>
-    <t>TC_G1_5</t>
-  </si>
-  <si>
     <t>Drumloop (4/4 Takt; Metadaten ermittelt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einspielen des Musikstücks mit dem Einspielgerät </t>
-  </si>
-  <si>
-    <t>Musikstück (4/4 Takt; Metadaten ermittelt) mit anschließender Offbeat-Phase</t>
   </si>
   <si>
     <t>Drumloop (4/4 Takt; 
@@ -539,18 +494,6 @@
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät </t>
   </si>
   <si>
-    <t>BPM-Wert muss nach Übergang in Offbeat-Phase weiterhin angezeigt werden, Signalisierung von fehlender Messdaten muss erfolgen</t>
-  </si>
-  <si>
-    <t>Musikstück (4/4 Takt; Metadaten ermittelt)</t>
-  </si>
-  <si>
-    <t>US_G1_1\2\3\5\6</t>
-  </si>
-  <si>
-    <t>US_G1_3\6</t>
-  </si>
-  <si>
     <t>US_G1_1\3</t>
   </si>
   <si>
@@ -559,9 +502,6 @@
   <si>
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät, dabei immer wieder das Tempo über den Pitch-Fader verändern (von 60 bis 180 BPM)
 </t>
-  </si>
-  <si>
-    <t>Sobald TC_G1_2 erfüllt ist und die Musik stoppt, muss der Wert für 10 Sekunden auf dem großen Display angezeigt werden und anschließend kleingedruckt am Bildschirmrand angezeigt werden, die Live Anzeige muss auf 0,0 zurückgesetzt werden</t>
   </si>
   <si>
     <t>BPM-Wert darf maximal um +/- 2 BPM vom vom  Einspielgerät angezeigten Wert abweichen, muss sich innerhalb von 5 Sekunden aktualisieren</t>
@@ -579,11 +519,6 @@
 A_G1_9</t>
   </si>
   <si>
-    <t>A_G1_10
-A_G1_11
-A_G1_12</t>
-  </si>
-  <si>
     <t xml:space="preserve">BPM-Wert darf maximal 
 um +/- 2 BPM von 
 Metadaten abweichen
@@ -594,17 +529,11 @@
 </t>
   </si>
   <si>
-    <t>Siehe TC_G1_2, wenn dies erfüllt ist, Signal pausieren</t>
-  </si>
-  <si>
     <t xml:space="preserve"> LED muss im Takt blinken</t>
   </si>
   <si>
     <t xml:space="preserve">Einspielen des 4 Beat Drumloops mit dem Einspielgerät 
 </t>
-  </si>
-  <si>
-    <t>TC_G1_6</t>
   </si>
   <si>
     <r>
@@ -713,6 +642,9 @@
   </si>
   <si>
     <t>3.2</t>
+  </si>
+  <si>
+    <t>US_G1_1\2\3\5</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1129,44 +1061,41 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1183,10 +1112,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1488,15 +1413,15 @@
         <v>90</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A5" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="50" t="s">
-        <v>185</v>
+      <c r="B5" s="38" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="34.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
@@ -1515,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="6" customWidth="1"/>
@@ -1552,30 +1477,30 @@
     </row>
     <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>98</v>
       </c>
       <c r="C2" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>122</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>99</v>
@@ -1584,7 +1509,7 @@
         <v>103</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>25</v>
@@ -1593,12 +1518,12 @@
         <v>25</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>100</v>
@@ -1607,7 +1532,7 @@
         <v>104</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>25</v>
@@ -1616,12 +1541,12 @@
         <v>25</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>101</v>
@@ -1639,12 +1564,12 @@
         <v>25</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>102</v>
@@ -1662,34 +1587,11 @@
         <v>25</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>143</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="7" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D12" s="29"/>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D11" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1701,17 +1603,17 @@
           <x14:formula1>
             <xm:f>LookUp!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E3 E4:E15</xm:sqref>
+          <xm:sqref>E2:E14</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
             <xm:f>LookUp!$C$2:$C$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F3 F4:F15</xm:sqref>
+          <xm:sqref>F2:F14</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
-            <xm:f>Anforderungen!$A$2:$A$23</xm:f>
+            <xm:f>Anforderungen!$A$2:$A$19</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
         </x14:dataValidation>
@@ -1723,7 +1625,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
@@ -1768,13 +1670,13 @@
     </row>
     <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B2" s="34" t="s">
         <v>107</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>30</v>
@@ -1786,18 +1688,18 @@
         <v>25</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B3" s="34" t="s">
         <v>112</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>25</v>
@@ -1809,18 +1711,18 @@
         <v>25</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>25</v>
@@ -1832,18 +1734,18 @@
         <v>25</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>25</v>
@@ -1855,18 +1757,18 @@
         <v>25</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>25</v>
@@ -1878,18 +1780,18 @@
         <v>25</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B7" s="34" t="s">
         <v>105</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>25</v>
@@ -1901,18 +1803,18 @@
         <v>25</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>106</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>25</v>
@@ -1924,19 +1826,19 @@
         <v>25</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>142</v>
-      </c>
       <c r="D9" s="7" t="s">
         <v>25</v>
       </c>
@@ -1947,18 +1849,18 @@
         <v>25</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>25</v>
@@ -1970,99 +1872,7 @@
         <v>25</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B11" s="28" t="s">
-        <v>136</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2075,7 +1885,7 @@
           <x14:formula1>
             <xm:f>LookUp!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>C15:C22</xm:sqref>
+          <xm:sqref>C11:C18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
           <x14:formula1>
@@ -2083,35 +1893,35 @@
           </x14:formula1>
           <xm:sqref>H2:H19</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000004000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
           <x14:formula1>
-            <xm:f>'User Stories'!$A$2:$A$15</xm:f>
+            <xm:f>'Test Cases'!$A$3:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>G15:G22</xm:sqref>
+          <xm:sqref>I2:I19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
           <x14:formula1>
             <xm:f>LookUp!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D22</xm:sqref>
+          <xm:sqref>D2:D18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000002000000}">
           <x14:formula1>
             <xm:f>LookUp!$D$2:$D$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E22</xm:sqref>
+          <xm:sqref>E2:E18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000003000000}">
           <x14:formula1>
             <xm:f>LookUp!$C$2:$C$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F22</xm:sqref>
+          <xm:sqref>F2:F18</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000005000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000004000000}">
           <x14:formula1>
-            <xm:f>'Test Cases'!$A$3:$A$7</xm:f>
+            <xm:f>'User Stories'!$A$2:$A$14</xm:f>
           </x14:formula1>
-          <xm:sqref>I2:I19</xm:sqref>
+          <xm:sqref>G11:G18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2132,15 +1942,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="D2" s="13" t="s">
@@ -2154,15 +1964,15 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="48"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="14" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2245,7 +2055,7 @@
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="10"/>
       <c r="C9" s="12" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>70</v>
@@ -2267,11 +2077,11 @@
       <c r="C11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="42"/>
-      <c r="F11" s="43"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
@@ -2280,11 +2090,11 @@
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
+      <c r="D12" s="45" t="s">
+        <v>142</v>
+      </c>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
@@ -2293,9 +2103,9 @@
       <c r="C13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="46"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
@@ -2304,9 +2114,9 @@
       <c r="C14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="46"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
@@ -2315,9 +2125,9 @@
       <c r="C15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="46"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
@@ -2326,9 +2136,9 @@
       <c r="C16" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="46"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
@@ -2337,9 +2147,9 @@
       <c r="C17" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="46"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
@@ -2348,9 +2158,9 @@
       <c r="C18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="46"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="49"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2406,247 +2216,221 @@
     </row>
     <row r="2" spans="1:8" s="29" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="E2" s="31" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="28"/>
       <c r="G2" s="28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="29" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="28" t="s">
         <v>156</v>
-      </c>
-      <c r="B3" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>164</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>177</v>
       </c>
       <c r="E3" s="31" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="28"/>
       <c r="G3" s="28" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="29" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="28" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="E4" s="31" t="s">
         <v>25</v>
       </c>
       <c r="F4" s="28"/>
       <c r="G4" s="28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="29" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>158</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>180</v>
       </c>
       <c r="E5" s="31" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="28"/>
       <c r="G5" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="H5" s="28"/>
-    </row>
-    <row r="6" spans="1:8" s="29" customFormat="1" ht="105" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
-        <v>159</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>165</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28" t="s">
-        <v>137</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" s="29" customFormat="1" ht="195" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>166</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>179</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="H7" s="28" t="s">
-        <v>147</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="H5" s="28" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6" s="9"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6" s="30"/>
+    </row>
+    <row r="7" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7"/>
+      <c r="B7" s="49" t="s">
+        <v>160</v>
+      </c>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="30"/>
     </row>
     <row r="8" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8" s="9"/>
-      <c r="F8"/>
-      <c r="G8"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
       <c r="H8" s="30"/>
     </row>
     <row r="9" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
-      <c r="B9" s="38" t="s">
-        <v>183</v>
-      </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
       <c r="H9" s="30"/>
     </row>
     <row r="10" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
       <c r="H10" s="30"/>
     </row>
     <row r="11" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
       <c r="H11" s="30"/>
     </row>
     <row r="12" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
       <c r="H12" s="30"/>
     </row>
     <row r="13" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="48"/>
       <c r="H13" s="30"/>
     </row>
     <row r="14" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="30"/>
     </row>
     <row r="15" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
       <c r="H15" s="30"/>
     </row>
     <row r="16" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16" s="9"/>
+      <c r="F16"/>
+      <c r="G16"/>
       <c r="H16" s="30"/>
     </row>
     <row r="17" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="30"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17" s="9"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17" s="33"/>
     </row>
     <row r="18" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
@@ -2656,7 +2440,7 @@
       <c r="E18" s="9"/>
       <c r="F18"/>
       <c r="G18"/>
-      <c r="H18" s="30"/>
+      <c r="H18" s="33"/>
     </row>
     <row r="19" spans="1:8" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19"/>
@@ -2670,7 +2454,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B9:G17"/>
+    <mergeCell ref="B7:G15"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -2682,13 +2466,13 @@
           <x14:formula1>
             <xm:f>LookUp!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E7</xm:sqref>
+          <xm:sqref>E2:E5</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
-            <xm:f>Anforderungen!$A$2:$A$23</xm:f>
+            <xm:f>Anforderungen!$A$2:$A$19</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G7</xm:sqref>
+          <xm:sqref>G2:G5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>